<commit_message>
allow it to work when NA's are present
</commit_message>
<xml_diff>
--- a/tests/testthat/data/coord_test.xlsx
+++ b/tests/testthat/data/coord_test.xlsx
@@ -462,9 +462,7 @@
       <c r="A4" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="2" t="n">
-        <v>39.9891</v>
-      </c>
+      <c r="B4" s="2"/>
       <c r="C4" s="2" t="n">
         <v>-79.5523</v>
       </c>

</xml_diff>